<commit_message>
fix: corrected export to excel (handling % sign)
</commit_message>
<xml_diff>
--- a/data/raw/Reference_Table.xlsx
+++ b/data/raw/Reference_Table.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/edoardociato/02_Work/TennisAnalytics_Master/TennisAnalyticsV3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/edoardociato/02_Work/TennisAnalytics_Master/TennisAnalyticsV3/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CCFCAFA-C5CD-AA44-8FF1-5D9262606F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF04B54A-C7BB-0D41-B0F3-01E12A549376}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4300" yWindow="780" windowWidth="29900" windowHeight="21460" xr2:uid="{589F79FF-B3DF-4A72-A764-0CD71D5A19DC}"/>
   </bookViews>
@@ -275,12 +275,6 @@
     <t>IO_Wnr%</t>
   </si>
   <si>
-    <t>DTL_Wnr%</t>
-  </si>
-  <si>
-    <t>DTL_Wnr%.1</t>
-  </si>
-  <si>
     <t>Ratio Winners / Unforced</t>
   </si>
   <si>
@@ -404,12 +398,6 @@
     <t>Categories</t>
   </si>
   <si>
-    <t>Down the Line Winners</t>
-  </si>
-  <si>
-    <t>Down the Line Winners 1st</t>
-  </si>
-  <si>
     <t>reference_table</t>
   </si>
   <si>
@@ -474,6 +462,18 @@
   </si>
   <si>
     <t>2nd Wide Speed</t>
+  </si>
+  <si>
+    <t>DTL_Wnr%_FH</t>
+  </si>
+  <si>
+    <t>DTL_Wnr%_BH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backhand Down the Line Winners </t>
+  </si>
+  <si>
+    <t>Forehand Down the Line Winners</t>
   </si>
 </sst>
 </file>
@@ -677,7 +677,7 @@
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>102046</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>88</xdr:row>
       <xdr:rowOff>106681</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -721,8 +721,8 @@
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>386286</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>164104</xdr:rowOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>133623</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -765,8 +765,8 @@
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>426720</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>174126</xdr:rowOff>
+      <xdr:row>83</xdr:row>
+      <xdr:rowOff>112562</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -809,8 +809,8 @@
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>298706</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>40368</xdr:rowOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>91356</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -853,7 +853,7 @@
     <xdr:to>
       <xdr:col>31</xdr:col>
       <xdr:colOff>17699</xdr:colOff>
-      <xdr:row>56</xdr:row>
+      <xdr:row>72</xdr:row>
       <xdr:rowOff>80422</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -892,7 +892,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4CF2A204-07DE-4E13-A729-0914269FED17}" name="Table1" displayName="Table1" ref="A2:K61" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
-  <autoFilter ref="A2:K61" xr:uid="{4CF2A204-07DE-4E13-A729-0914269FED17}"/>
+  <autoFilter ref="A2:K61" xr:uid="{4CF2A204-07DE-4E13-A729-0914269FED17}">
+    <filterColumn colId="10">
+      <filters>
+        <filter val="0"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{DCA3A328-43A0-4C5B-8661-6C80084ACF61}" name="variable"/>
     <tableColumn id="4" xr3:uid="{6999234A-287D-4816-9670-BB216BACB7D2}" name="Parity"/>
@@ -1256,31 +1262,31 @@
         <v>3</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="M2" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1303,10 +1309,10 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I3" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -1318,7 +1324,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1341,10 +1347,10 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I4" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -1356,7 +1362,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1379,10 +1385,10 @@
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I5" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J5">
         <v>0</v>
@@ -1394,7 +1400,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -1417,10 +1423,10 @@
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I6" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -1432,7 +1438,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1455,10 +1461,10 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I7" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J7">
         <v>0</v>
@@ -1470,7 +1476,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -1493,10 +1499,10 @@
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I8" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J8">
         <v>0</v>
@@ -1505,10 +1511,10 @@
         <v>1</v>
       </c>
       <c r="M8" s="8" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1531,10 +1537,10 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I9" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -1566,10 +1572,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I10" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J10">
         <v>0</v>
@@ -1586,7 +1592,7 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D11" t="s">
         <v>5</v>
@@ -1601,10 +1607,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I11" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J11">
         <v>0</v>
@@ -1636,10 +1642,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I12" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J12">
         <v>0</v>
@@ -1671,10 +1677,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I13" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J13">
         <v>0</v>
@@ -1691,7 +1697,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D14" t="s">
         <v>5</v>
@@ -1706,10 +1712,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I14" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J14">
         <v>0</v>
@@ -1726,7 +1732,7 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D15" t="s">
         <v>5</v>
@@ -1741,10 +1747,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I15" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J15">
         <v>0</v>
@@ -1753,7 +1759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1776,10 +1782,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="I16" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J16">
         <v>0</v>
@@ -1788,7 +1794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -1811,10 +1817,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I17" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J17">
         <v>0</v>
@@ -1823,7 +1829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -1846,10 +1852,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I18" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J18">
         <v>0</v>
@@ -1858,7 +1864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>34</v>
       </c>
@@ -1881,10 +1887,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="I19" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J19">
         <v>0</v>
@@ -1893,7 +1899,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -1916,10 +1922,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="I20" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J20">
         <v>0</v>
@@ -1928,7 +1934,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -1951,10 +1957,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="I21" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J21">
         <v>0</v>
@@ -1963,7 +1969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -1986,10 +1992,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="I22" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J22">
         <v>0</v>
@@ -1998,7 +2004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -2021,10 +2027,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I23" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J23">
         <v>0</v>
@@ -2033,7 +2039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>45</v>
       </c>
@@ -2056,10 +2062,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="I24" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J24">
         <v>0</v>
@@ -2068,7 +2074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>47</v>
       </c>
@@ -2091,10 +2097,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="I25" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J25">
         <v>0</v>
@@ -2103,7 +2109,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>49</v>
       </c>
@@ -2126,10 +2132,10 @@
         <v>1</v>
       </c>
       <c r="H26" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I26" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J26">
         <v>0</v>
@@ -2138,7 +2144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>52</v>
       </c>
@@ -2161,10 +2167,10 @@
         <v>1</v>
       </c>
       <c r="H27" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I27" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J27">
         <v>0</v>
@@ -2173,7 +2179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>54</v>
       </c>
@@ -2196,10 +2202,10 @@
         <v>1</v>
       </c>
       <c r="H28" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I28" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J28">
         <v>0</v>
@@ -2208,7 +2214,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>56</v>
       </c>
@@ -2231,10 +2237,10 @@
         <v>1</v>
       </c>
       <c r="H29" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="I29" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J29">
         <v>0</v>
@@ -2243,7 +2249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>58</v>
       </c>
@@ -2266,10 +2272,10 @@
         <v>1</v>
       </c>
       <c r="H30" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I30" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J30">
         <v>0</v>
@@ -2278,7 +2284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>60</v>
       </c>
@@ -2301,10 +2307,10 @@
         <v>1</v>
       </c>
       <c r="H31" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I31" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J31">
         <v>0</v>
@@ -2313,7 +2319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>62</v>
       </c>
@@ -2336,10 +2342,10 @@
         <v>1</v>
       </c>
       <c r="H32" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I32" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J32">
         <v>0</v>
@@ -2348,7 +2354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -2371,10 +2377,10 @@
         <v>1</v>
       </c>
       <c r="H33" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="I33" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J33">
         <v>0</v>
@@ -2383,7 +2389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>67</v>
       </c>
@@ -2406,10 +2412,10 @@
         <v>1</v>
       </c>
       <c r="H34" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="I34" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J34">
         <v>0</v>
@@ -2418,7 +2424,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>69</v>
       </c>
@@ -2441,10 +2447,10 @@
         <v>1</v>
       </c>
       <c r="H35" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I35" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J35">
         <v>0</v>
@@ -2453,7 +2459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>72</v>
       </c>
@@ -2476,10 +2482,10 @@
         <v>1</v>
       </c>
       <c r="H36" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I36" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J36">
         <v>0</v>
@@ -2488,7 +2494,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>74</v>
       </c>
@@ -2511,10 +2517,10 @@
         <v>1</v>
       </c>
       <c r="H37" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I37" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J37">
         <v>0</v>
@@ -2523,7 +2529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>76</v>
       </c>
@@ -2546,10 +2552,10 @@
         <v>1</v>
       </c>
       <c r="H38" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I38" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J38">
         <v>0</v>
@@ -2558,7 +2564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>78</v>
       </c>
@@ -2581,10 +2587,10 @@
         <v>1</v>
       </c>
       <c r="H39" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I39" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J39">
         <v>0</v>
@@ -2593,15 +2599,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>79</v>
+        <v>142</v>
       </c>
       <c r="B40">
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
       <c r="D40" t="s">
         <v>70</v>
@@ -2616,10 +2622,10 @@
         <v>1</v>
       </c>
       <c r="H40" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I40" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J40">
         <v>0</v>
@@ -2628,15 +2634,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>80</v>
+        <v>143</v>
       </c>
       <c r="B41">
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="D41" t="s">
         <v>70</v>
@@ -2651,10 +2657,10 @@
         <v>1</v>
       </c>
       <c r="H41" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I41" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J41">
         <v>0</v>
@@ -2665,13 +2671,13 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B42">
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D42" t="s">
         <v>70</v>
@@ -2686,10 +2692,10 @@
         <v>1</v>
       </c>
       <c r="H42" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="I42" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J42">
         <v>0</v>
@@ -2698,15 +2704,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B43">
         <v>0</v>
       </c>
       <c r="C43" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D43" t="s">
         <v>43</v>
@@ -2721,10 +2727,10 @@
         <v>1</v>
       </c>
       <c r="H43" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I43" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J43">
         <v>0</v>
@@ -2733,15 +2739,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B44">
         <v>0</v>
       </c>
       <c r="C44" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D44" t="s">
         <v>43</v>
@@ -2756,10 +2762,10 @@
         <v>1</v>
       </c>
       <c r="H44" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I44" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J44">
         <v>0</v>
@@ -2768,15 +2774,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B45">
         <v>0</v>
       </c>
       <c r="C45" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D45" t="s">
         <v>43</v>
@@ -2791,10 +2797,10 @@
         <v>1</v>
       </c>
       <c r="H45" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I45" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J45">
         <v>0</v>
@@ -2805,13 +2811,13 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B46">
         <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D46" t="s">
         <v>63</v>
@@ -2826,10 +2832,10 @@
         <v>1</v>
       </c>
       <c r="H46" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I46" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J46">
         <v>0</v>
@@ -2840,13 +2846,13 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B47">
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D47" t="s">
         <v>63</v>
@@ -2861,10 +2867,10 @@
         <v>1</v>
       </c>
       <c r="H47" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I47" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J47">
         <v>0</v>
@@ -2873,15 +2879,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B48">
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D48" t="s">
         <v>63</v>
@@ -2896,10 +2902,10 @@
         <v>1</v>
       </c>
       <c r="H48" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I48" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J48">
         <v>0</v>
@@ -2908,15 +2914,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B49">
         <v>1</v>
       </c>
       <c r="C49" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D49" t="s">
         <v>63</v>
@@ -2931,10 +2937,10 @@
         <v>1</v>
       </c>
       <c r="H49" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I49" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J49">
         <v>0</v>
@@ -2943,15 +2949,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B50">
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D50" t="s">
         <v>63</v>
@@ -2966,10 +2972,10 @@
         <v>1</v>
       </c>
       <c r="H50" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="I50" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J50">
         <v>0</v>
@@ -2978,15 +2984,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B51">
         <v>1</v>
       </c>
       <c r="C51" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D51" t="s">
         <v>63</v>
@@ -3001,10 +3007,10 @@
         <v>1</v>
       </c>
       <c r="H51" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I51" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J51">
         <v>0</v>
@@ -3015,13 +3021,13 @@
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B52">
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D52" t="s">
         <v>63</v>
@@ -3036,10 +3042,10 @@
         <v>1</v>
       </c>
       <c r="H52" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I52" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J52">
         <v>0</v>
@@ -3048,15 +3054,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B53">
         <v>-1</v>
       </c>
       <c r="C53" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D53" t="s">
         <v>50</v>
@@ -3071,7 +3077,7 @@
         <v>0</v>
       </c>
       <c r="H53" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="J53">
         <v>1</v>
@@ -3080,15 +3086,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B54">
         <v>1</v>
       </c>
       <c r="C54" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D54" t="s">
         <v>50</v>
@@ -3103,7 +3109,7 @@
         <v>0</v>
       </c>
       <c r="H54" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="J54">
         <v>1</v>
@@ -3112,15 +3118,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B55">
         <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D55" t="s">
         <v>50</v>
@@ -3135,7 +3141,7 @@
         <v>0</v>
       </c>
       <c r="H55" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="J55">
         <v>1</v>
@@ -3144,15 +3150,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B56">
         <v>-1</v>
       </c>
       <c r="C56" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D56" t="s">
         <v>50</v>
@@ -3167,7 +3173,7 @@
         <v>0</v>
       </c>
       <c r="H56" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="J56">
         <v>1</v>
@@ -3176,15 +3182,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B57">
         <v>0</v>
       </c>
       <c r="C57" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D57" t="s">
         <v>43</v>
@@ -3199,7 +3205,7 @@
         <v>1</v>
       </c>
       <c r="H57" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J57">
         <v>1</v>
@@ -3208,15 +3214,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B58">
         <v>0</v>
       </c>
       <c r="C58" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D58" t="s">
         <v>43</v>
@@ -3231,7 +3237,7 @@
         <v>1</v>
       </c>
       <c r="H58" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J58">
         <v>1</v>
@@ -3240,15 +3246,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B59">
         <v>0</v>
       </c>
       <c r="C59" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D59" t="s">
         <v>43</v>
@@ -3263,7 +3269,7 @@
         <v>1</v>
       </c>
       <c r="H59" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J59">
         <v>1</v>
@@ -3272,15 +3278,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B60">
         <v>0</v>
       </c>
       <c r="C60" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D60" t="s">
         <v>43</v>
@@ -3295,7 +3301,7 @@
         <v>1</v>
       </c>
       <c r="H60" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J60">
         <v>1</v>
@@ -3304,15 +3310,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B61">
         <v>0</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D61" t="s">
         <v>43</v>
@@ -3327,7 +3333,7 @@
         <v>1</v>
       </c>
       <c r="H61" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J61">
         <v>1</v>

</xml_diff>

<commit_message>
feat: included serve direction
</commit_message>
<xml_diff>
--- a/data/raw/Reference_Table.xlsx
+++ b/data/raw/Reference_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/edoardociato/02_Work/TennisAnalytics_Master/TennisAnalyticsV3/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F9569D1-D467-FA48-95B0-B542A76E6A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F56BEF-A284-9D4A-8591-456A56C73B63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4300" yWindow="780" windowWidth="29900" windowHeight="21460" xr2:uid="{589F79FF-B3DF-4A72-A764-0CD71D5A19DC}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="163">
   <si>
     <t>Description</t>
   </si>
@@ -353,42 +353,6 @@
     <t>very_deep</t>
   </si>
   <si>
-    <t>Return unforced %</t>
-  </si>
-  <si>
-    <t>unforced</t>
-  </si>
-  <si>
-    <t>Cross court %</t>
-  </si>
-  <si>
-    <t>crosscourt</t>
-  </si>
-  <si>
-    <t>Down middle %</t>
-  </si>
-  <si>
-    <t>down_middle</t>
-  </si>
-  <si>
-    <t>Down the Line %</t>
-  </si>
-  <si>
-    <t>down_the_line</t>
-  </si>
-  <si>
-    <t>Inside Out %</t>
-  </si>
-  <si>
-    <t>inside_out</t>
-  </si>
-  <si>
-    <t>Inside In%</t>
-  </si>
-  <si>
-    <t>inside_in</t>
-  </si>
-  <si>
     <t>Chart</t>
   </si>
   <si>
@@ -464,16 +428,103 @@
     <t>2nd Wide Speed</t>
   </si>
   <si>
-    <t>DTL_Wnr%_FH</t>
-  </si>
-  <si>
-    <t>DTL_Wnr%_BH</t>
-  </si>
-  <si>
     <t xml:space="preserve">Backhand Down the Line Winners </t>
   </si>
   <si>
     <t>Forehand Down the Line Winners</t>
+  </si>
+  <si>
+    <t>Serve deuce side wide %</t>
+  </si>
+  <si>
+    <t>Serve deuce side middle %</t>
+  </si>
+  <si>
+    <t>Serve deuce side t %</t>
+  </si>
+  <si>
+    <t>Serve ad side wide %</t>
+  </si>
+  <si>
+    <t>Serve ad side middle %</t>
+  </si>
+  <si>
+    <t>Serve ad side t %</t>
+  </si>
+  <si>
+    <t>ad_t</t>
+  </si>
+  <si>
+    <t>ad_middle</t>
+  </si>
+  <si>
+    <t>ad_wide</t>
+  </si>
+  <si>
+    <t>deuce_t</t>
+  </si>
+  <si>
+    <t>deuce_middle</t>
+  </si>
+  <si>
+    <t>deuce_wide</t>
+  </si>
+  <si>
+    <t>mcp_m_stats_servedirection</t>
+  </si>
+  <si>
+    <t>DTL_Wnr%</t>
+  </si>
+  <si>
+    <t>DTL_Wnr%.1</t>
+  </si>
+  <si>
+    <t>crosscourt_FH</t>
+  </si>
+  <si>
+    <t>down_middle_FH</t>
+  </si>
+  <si>
+    <t>down_the_line_FH</t>
+  </si>
+  <si>
+    <t>inside_out_FH</t>
+  </si>
+  <si>
+    <t>inside_in_FH</t>
+  </si>
+  <si>
+    <t>crosscourt_BH</t>
+  </si>
+  <si>
+    <t>down_middle_BH</t>
+  </si>
+  <si>
+    <t>down_the_line_BH</t>
+  </si>
+  <si>
+    <t>Forehand Cross court %</t>
+  </si>
+  <si>
+    <t>Forehand Down middle %</t>
+  </si>
+  <si>
+    <t>Forehand Down the Line %</t>
+  </si>
+  <si>
+    <t>Forehand inside In%</t>
+  </si>
+  <si>
+    <t>Backhand Cross court %</t>
+  </si>
+  <si>
+    <t>Backhand Down middle %</t>
+  </si>
+  <si>
+    <t>Backhand Down the Line %</t>
+  </si>
+  <si>
+    <t>Forehand inside Out %</t>
   </si>
 </sst>
 </file>
@@ -677,7 +728,7 @@
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>102046</xdr:colOff>
-      <xdr:row>90</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>106681</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -721,8 +772,8 @@
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>386286</xdr:colOff>
-      <xdr:row>69</xdr:row>
-      <xdr:rowOff>164103</xdr:rowOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>164104</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -765,7 +816,7 @@
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>426720</xdr:colOff>
-      <xdr:row>85</xdr:row>
+      <xdr:row>66</xdr:row>
       <xdr:rowOff>174126</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -809,8 +860,8 @@
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>298706</xdr:colOff>
-      <xdr:row>73</xdr:row>
-      <xdr:rowOff>91356</xdr:rowOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>40368</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -853,8 +904,8 @@
     <xdr:to>
       <xdr:col>31</xdr:col>
       <xdr:colOff>17699</xdr:colOff>
-      <xdr:row>75</xdr:row>
-      <xdr:rowOff>80421</xdr:rowOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>80422</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -891,14 +942,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4CF2A204-07DE-4E13-A729-0914269FED17}" name="Table1" displayName="Table1" ref="A2:K61" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
-  <autoFilter ref="A2:K61" xr:uid="{4CF2A204-07DE-4E13-A729-0914269FED17}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="Rally"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4CF2A204-07DE-4E13-A729-0914269FED17}" name="Table1" displayName="Table1" ref="A2:K71" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
+  <autoFilter ref="A2:K71" xr:uid="{4CF2A204-07DE-4E13-A729-0914269FED17}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{DCA3A328-43A0-4C5B-8661-6C80084ACF61}" name="variable"/>
     <tableColumn id="4" xr3:uid="{6999234A-287D-4816-9670-BB216BACB7D2}" name="Parity"/>
@@ -1233,7 +1278,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C70B48F9-3C73-4604-B662-B76B4FE5C262}">
-  <dimension ref="A2:M61"/>
+  <dimension ref="A2:M69"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" customWidth="1"/>
@@ -1265,28 +1310,28 @@
         <v>81</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>130</v>
-      </c>
       <c r="J2" s="2" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>80</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1309,10 +1354,10 @@
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="I3" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -1324,7 +1369,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1347,10 +1392,10 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="I4" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -1362,7 +1407,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1385,10 +1430,10 @@
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="I5" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="J5">
         <v>0</v>
@@ -1400,7 +1445,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -1423,10 +1468,10 @@
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="I6" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -1438,7 +1483,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1461,10 +1506,10 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="I7" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="J7">
         <v>0</v>
@@ -1476,7 +1521,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -1499,10 +1544,10 @@
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="I8" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="J8">
         <v>0</v>
@@ -1514,7 +1559,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1537,10 +1582,10 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="I9" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -1549,7 +1594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1572,10 +1617,10 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="I10" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J10">
         <v>0</v>
@@ -1584,7 +1629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1592,7 +1637,7 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="D11" t="s">
         <v>5</v>
@@ -1607,10 +1652,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="I11" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J11">
         <v>0</v>
@@ -1619,7 +1664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1642,10 +1687,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="I12" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J12">
         <v>0</v>
@@ -1654,7 +1699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1677,10 +1722,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="I13" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J13">
         <v>0</v>
@@ -1689,7 +1734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -1697,7 +1742,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="D14" t="s">
         <v>5</v>
@@ -1712,10 +1757,10 @@
         <v>0</v>
       </c>
       <c r="H14" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="I14" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J14">
         <v>0</v>
@@ -1724,7 +1769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -1732,7 +1777,7 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="D15" t="s">
         <v>5</v>
@@ -1747,10 +1792,10 @@
         <v>0</v>
       </c>
       <c r="H15" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="I15" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J15">
         <v>0</v>
@@ -1759,7 +1804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1782,10 +1827,10 @@
         <v>0</v>
       </c>
       <c r="H16" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="I16" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J16">
         <v>0</v>
@@ -1794,7 +1839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -1817,10 +1862,10 @@
         <v>0</v>
       </c>
       <c r="H17" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="I17" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J17">
         <v>0</v>
@@ -1829,7 +1874,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -1852,10 +1897,10 @@
         <v>0</v>
       </c>
       <c r="H18" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="I18" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J18">
         <v>0</v>
@@ -1864,7 +1909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>34</v>
       </c>
@@ -1887,10 +1932,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I19" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J19">
         <v>0</v>
@@ -1899,7 +1944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>36</v>
       </c>
@@ -1922,10 +1967,10 @@
         <v>0</v>
       </c>
       <c r="H20" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I20" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J20">
         <v>0</v>
@@ -1934,7 +1979,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>38</v>
       </c>
@@ -1957,10 +2002,10 @@
         <v>0</v>
       </c>
       <c r="H21" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I21" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J21">
         <v>0</v>
@@ -1969,7 +2014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -1992,10 +2037,10 @@
         <v>0</v>
       </c>
       <c r="H22" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I22" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J22">
         <v>0</v>
@@ -2004,7 +2049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>42</v>
       </c>
@@ -2027,10 +2072,10 @@
         <v>0</v>
       </c>
       <c r="H23" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="I23" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J23">
         <v>0</v>
@@ -2039,7 +2084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>45</v>
       </c>
@@ -2062,10 +2107,10 @@
         <v>0</v>
       </c>
       <c r="H24" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I24" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J24">
         <v>0</v>
@@ -2074,7 +2119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>47</v>
       </c>
@@ -2097,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="s">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="I25" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J25">
         <v>0</v>
@@ -2109,7 +2154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>49</v>
       </c>
@@ -2132,10 +2177,10 @@
         <v>1</v>
       </c>
       <c r="H26" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="I26" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="J26">
         <v>0</v>
@@ -2144,7 +2189,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>52</v>
       </c>
@@ -2167,10 +2212,10 @@
         <v>1</v>
       </c>
       <c r="H27" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="I27" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="J27">
         <v>0</v>
@@ -2179,7 +2224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>54</v>
       </c>
@@ -2202,10 +2247,10 @@
         <v>1</v>
       </c>
       <c r="H28" t="s">
-        <v>128</v>
+        <v>116</v>
       </c>
       <c r="I28" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J28">
         <v>0</v>
@@ -2214,7 +2259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>56</v>
       </c>
@@ -2237,10 +2282,10 @@
         <v>1</v>
       </c>
       <c r="H29" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="I29" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J29">
         <v>0</v>
@@ -2249,7 +2294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>58</v>
       </c>
@@ -2272,10 +2317,10 @@
         <v>1</v>
       </c>
       <c r="H30" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="I30" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J30">
         <v>0</v>
@@ -2284,7 +2329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>60</v>
       </c>
@@ -2307,10 +2352,10 @@
         <v>1</v>
       </c>
       <c r="H31" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="I31" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J31">
         <v>0</v>
@@ -2319,7 +2364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>62</v>
       </c>
@@ -2342,10 +2387,10 @@
         <v>1</v>
       </c>
       <c r="H32" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="I32" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J32">
         <v>0</v>
@@ -2354,7 +2399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -2377,10 +2422,10 @@
         <v>1</v>
       </c>
       <c r="H33" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I33" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J33">
         <v>0</v>
@@ -2389,7 +2434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>67</v>
       </c>
@@ -2412,10 +2457,10 @@
         <v>1</v>
       </c>
       <c r="H34" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="I34" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J34">
         <v>0</v>
@@ -2447,10 +2492,10 @@
         <v>1</v>
       </c>
       <c r="H35" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="I35" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J35">
         <v>0</v>
@@ -2482,10 +2527,10 @@
         <v>1</v>
       </c>
       <c r="H36" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="I36" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J36">
         <v>0</v>
@@ -2517,10 +2562,10 @@
         <v>1</v>
       </c>
       <c r="H37" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="I37" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J37">
         <v>0</v>
@@ -2552,10 +2597,10 @@
         <v>1</v>
       </c>
       <c r="H38" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="I38" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J38">
         <v>0</v>
@@ -2587,10 +2632,10 @@
         <v>1</v>
       </c>
       <c r="H39" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="I39" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J39">
         <v>0</v>
@@ -2601,13 +2646,13 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B40">
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D40" t="s">
         <v>70</v>
@@ -2622,10 +2667,10 @@
         <v>1</v>
       </c>
       <c r="H40" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="I40" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J40">
         <v>0</v>
@@ -2636,13 +2681,13 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B41">
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="D41" t="s">
         <v>70</v>
@@ -2657,10 +2702,10 @@
         <v>1</v>
       </c>
       <c r="H41" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="I41" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J41">
         <v>0</v>
@@ -2692,10 +2737,10 @@
         <v>1</v>
       </c>
       <c r="H42" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="I42" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J42">
         <v>0</v>
@@ -2704,7 +2749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>82</v>
       </c>
@@ -2712,7 +2757,7 @@
         <v>0</v>
       </c>
       <c r="C43" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="D43" t="s">
         <v>43</v>
@@ -2727,10 +2772,10 @@
         <v>1</v>
       </c>
       <c r="H43" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="I43" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J43">
         <v>0</v>
@@ -2739,7 +2784,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>84</v>
       </c>
@@ -2762,10 +2807,10 @@
         <v>1</v>
       </c>
       <c r="H44" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="I44" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J44">
         <v>0</v>
@@ -2774,7 +2819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>86</v>
       </c>
@@ -2797,10 +2842,10 @@
         <v>1</v>
       </c>
       <c r="H45" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="I45" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J45">
         <v>0</v>
@@ -2809,7 +2854,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>87</v>
       </c>
@@ -2817,7 +2862,7 @@
         <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="D46" t="s">
         <v>63</v>
@@ -2832,10 +2877,10 @@
         <v>1</v>
       </c>
       <c r="H46" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="I46" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J46">
         <v>0</v>
@@ -2844,7 +2889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>89</v>
       </c>
@@ -2867,10 +2912,10 @@
         <v>1</v>
       </c>
       <c r="H47" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="I47" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J47">
         <v>0</v>
@@ -2879,7 +2924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>91</v>
       </c>
@@ -2902,10 +2947,10 @@
         <v>1</v>
       </c>
       <c r="H48" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="I48" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J48">
         <v>0</v>
@@ -2914,7 +2959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>93</v>
       </c>
@@ -2937,10 +2982,10 @@
         <v>1</v>
       </c>
       <c r="H49" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="I49" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J49">
         <v>0</v>
@@ -2949,7 +2994,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>94</v>
       </c>
@@ -2957,7 +3002,7 @@
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="D50" t="s">
         <v>63</v>
@@ -2972,10 +3017,10 @@
         <v>1</v>
       </c>
       <c r="H50" t="s">
-        <v>124</v>
+        <v>112</v>
       </c>
       <c r="I50" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J50">
         <v>0</v>
@@ -2984,7 +3029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>96</v>
       </c>
@@ -3007,10 +3052,10 @@
         <v>1</v>
       </c>
       <c r="H51" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="I51" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="J51">
         <v>0</v>
@@ -3019,7 +3064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>98</v>
       </c>
@@ -3042,10 +3087,10 @@
         <v>1</v>
       </c>
       <c r="H52" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="I52" t="s">
-        <v>131</v>
+        <v>119</v>
       </c>
       <c r="J52">
         <v>0</v>
@@ -3054,7 +3099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>100</v>
       </c>
@@ -3077,7 +3122,7 @@
         <v>0</v>
       </c>
       <c r="H53" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="J53">
         <v>1</v>
@@ -3086,7 +3131,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>102</v>
       </c>
@@ -3109,7 +3154,7 @@
         <v>0</v>
       </c>
       <c r="H54" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="J54">
         <v>1</v>
@@ -3118,7 +3163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>104</v>
       </c>
@@ -3141,7 +3186,7 @@
         <v>0</v>
       </c>
       <c r="H55" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="J55">
         <v>1</v>
@@ -3150,30 +3195,30 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="B56">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C56" t="s">
-        <v>105</v>
+        <v>155</v>
       </c>
       <c r="D56" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E56">
         <v>0</v>
       </c>
       <c r="F56" s="6">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H56" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="J56">
         <v>1</v>
@@ -3182,15 +3227,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>108</v>
+        <v>148</v>
       </c>
       <c r="B57">
         <v>0</v>
       </c>
       <c r="C57" t="s">
-        <v>107</v>
+        <v>156</v>
       </c>
       <c r="D57" t="s">
         <v>43</v>
@@ -3199,13 +3244,13 @@
         <v>0</v>
       </c>
       <c r="F57" s="6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G57">
         <v>1</v>
       </c>
       <c r="H57" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="J57">
         <v>1</v>
@@ -3214,15 +3259,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>110</v>
+        <v>149</v>
       </c>
       <c r="B58">
         <v>0</v>
       </c>
       <c r="C58" t="s">
-        <v>109</v>
+        <v>157</v>
       </c>
       <c r="D58" t="s">
         <v>43</v>
@@ -3231,13 +3276,13 @@
         <v>0</v>
       </c>
       <c r="F58" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G58">
         <v>1</v>
       </c>
       <c r="H58" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="J58">
         <v>1</v>
@@ -3246,15 +3291,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>112</v>
+        <v>150</v>
       </c>
       <c r="B59">
         <v>0</v>
       </c>
       <c r="C59" t="s">
-        <v>111</v>
+        <v>162</v>
       </c>
       <c r="D59" t="s">
         <v>43</v>
@@ -3263,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="F59" s="6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G59">
         <v>1</v>
       </c>
       <c r="H59" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="J59">
         <v>1</v>
@@ -3278,15 +3323,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>114</v>
+        <v>151</v>
       </c>
       <c r="B60">
         <v>0</v>
       </c>
-      <c r="C60" t="s">
-        <v>113</v>
+      <c r="C60" s="4" t="s">
+        <v>158</v>
       </c>
       <c r="D60" t="s">
         <v>43</v>
@@ -3301,7 +3346,7 @@
         <v>1</v>
       </c>
       <c r="H60" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="J60">
         <v>1</v>
@@ -3310,15 +3355,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="B61">
         <v>0</v>
       </c>
-      <c r="C61" s="4" t="s">
-        <v>115</v>
+      <c r="C61" t="s">
+        <v>159</v>
       </c>
       <c r="D61" t="s">
         <v>43</v>
@@ -3327,18 +3372,274 @@
         <v>0</v>
       </c>
       <c r="F61" s="6">
+        <v>4</v>
+      </c>
+      <c r="G61">
+        <v>1</v>
+      </c>
+      <c r="H61" t="s">
+        <v>124</v>
+      </c>
+      <c r="J61">
+        <v>1</v>
+      </c>
+      <c r="K61">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>153</v>
+      </c>
+      <c r="B62">
+        <v>0</v>
+      </c>
+      <c r="C62" t="s">
+        <v>160</v>
+      </c>
+      <c r="D62" t="s">
+        <v>43</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+      <c r="F62" s="6">
         <v>6</v>
       </c>
-      <c r="G61">
-        <v>1</v>
-      </c>
-      <c r="H61" t="s">
+      <c r="G62">
+        <v>1</v>
+      </c>
+      <c r="H62" t="s">
+        <v>124</v>
+      </c>
+      <c r="J62">
+        <v>1</v>
+      </c>
+      <c r="K62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>154</v>
+      </c>
+      <c r="B63">
+        <v>0</v>
+      </c>
+      <c r="C63" t="s">
+        <v>161</v>
+      </c>
+      <c r="D63" t="s">
+        <v>43</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+      <c r="F63" s="6">
+        <v>5</v>
+      </c>
+      <c r="G63">
+        <v>1</v>
+      </c>
+      <c r="H63" t="s">
+        <v>124</v>
+      </c>
+      <c r="J63">
+        <v>1</v>
+      </c>
+      <c r="K63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>143</v>
+      </c>
+      <c r="B64">
+        <v>0</v>
+      </c>
+      <c r="C64" t="s">
+        <v>132</v>
+      </c>
+      <c r="D64" t="s">
+        <v>43</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+      <c r="F64" s="6">
+        <v>9</v>
+      </c>
+      <c r="G64">
+        <v>1</v>
+      </c>
+      <c r="H64" t="s">
+        <v>144</v>
+      </c>
+      <c r="J64">
+        <v>1</v>
+      </c>
+      <c r="K64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>142</v>
+      </c>
+      <c r="B65">
+        <v>0</v>
+      </c>
+      <c r="C65" t="s">
+        <v>133</v>
+      </c>
+      <c r="D65" t="s">
+        <v>43</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65" s="6">
+        <v>10</v>
+      </c>
+      <c r="G65">
+        <v>1</v>
+      </c>
+      <c r="H65" t="s">
+        <v>144</v>
+      </c>
+      <c r="J65">
+        <v>1</v>
+      </c>
+      <c r="K65">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>141</v>
+      </c>
+      <c r="B66">
+        <v>0</v>
+      </c>
+      <c r="C66" t="s">
+        <v>134</v>
+      </c>
+      <c r="D66" t="s">
+        <v>43</v>
+      </c>
+      <c r="E66">
+        <v>0</v>
+      </c>
+      <c r="F66" s="6">
+        <v>11</v>
+      </c>
+      <c r="G66">
+        <v>1</v>
+      </c>
+      <c r="H66" t="s">
+        <v>144</v>
+      </c>
+      <c r="J66">
+        <v>1</v>
+      </c>
+      <c r="K66">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>140</v>
+      </c>
+      <c r="B67">
+        <v>0</v>
+      </c>
+      <c r="C67" t="s">
+        <v>135</v>
+      </c>
+      <c r="D67" t="s">
+        <v>43</v>
+      </c>
+      <c r="E67">
+        <v>0</v>
+      </c>
+      <c r="F67" s="6">
+        <v>12</v>
+      </c>
+      <c r="G67">
+        <v>1</v>
+      </c>
+      <c r="H67" t="s">
+        <v>144</v>
+      </c>
+      <c r="J67">
+        <v>1</v>
+      </c>
+      <c r="K67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>139</v>
+      </c>
+      <c r="B68">
+        <v>0</v>
+      </c>
+      <c r="C68" t="s">
         <v>136</v>
       </c>
-      <c r="J61">
-        <v>1</v>
-      </c>
-      <c r="K61">
+      <c r="D68" t="s">
+        <v>43</v>
+      </c>
+      <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68" s="6">
+        <v>13</v>
+      </c>
+      <c r="G68">
+        <v>1</v>
+      </c>
+      <c r="H68" t="s">
+        <v>144</v>
+      </c>
+      <c r="J68">
+        <v>1</v>
+      </c>
+      <c r="K68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>138</v>
+      </c>
+      <c r="B69">
+        <v>0</v>
+      </c>
+      <c r="C69" t="s">
+        <v>137</v>
+      </c>
+      <c r="D69" t="s">
+        <v>43</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+      <c r="F69" s="6">
+        <v>14</v>
+      </c>
+      <c r="G69">
+        <v>1</v>
+      </c>
+      <c r="H69" t="s">
+        <v>144</v>
+      </c>
+      <c r="J69">
+        <v>1</v>
+      </c>
+      <c r="K69">
         <v>1</v>
       </c>
     </row>
@@ -3347,7 +3648,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M8" xr:uid="{A1296866-C643-430F-9178-AD2520CDAA44}">
       <formula1>$M$2:$M$8</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D61" xr:uid="{1643AB3D-26ED-4117-AB07-6DC5F748532F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D71" xr:uid="{1643AB3D-26ED-4117-AB07-6DC5F748532F}">
       <formula1>$M$3:$M$8</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>